<commit_message>
Complete Solvix Phase 1 MVP: guardrail hardening, PR revision, task dashboard
Accumulates the remaining MVP work: assertion-gaming/weak-test-coverage
detection and dangerous-ops confirmation hardening in the retry loop,
conversational PR revision (SLX-D3: `solvix revise <pr_number>` reuses the
full guarded pipeline against a PR's existing branch and fetched human
feedback), and a CLI task-outcomes dashboard (SLX-D4: `solvix history` /
`solvix stats` backed by a new SQLite task_history.db per repo).

Also fixes two bugs found while smoke-testing D3/D4 against the real repo:
`pyproject.toml`'s package discovery was missing the `review`/`memory`
packages (the installed `solvix` CLI couldn't import them), and the
git-apply/patch fallback added for D3 was leaving `.orig` backup files in
the target repo's working tree.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Solvix-Full-Story-Backlog.xlsx
+++ b/docs/Solvix-Full-Story-Backlog.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Phase Overview" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Backlog!$A$1:$K$38</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Backlog!$A$1:$K$41</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="250">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -171,273 +171,273 @@
     <t xml:space="preserve">epic:requirement-understanding, priority:should, type:feature, phase:1</t>
   </si>
   <si>
+    <t xml:space="preserve">SLX-B3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Produce a reviewable task plan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a tech lead, I want the agent to break a larger requirement into a task plan I can review before it starts editing, so that I can catch scope issues early.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agent outputs an ordered plan (files to touch, approach) before any code is modified, and waits for approval if the task is flagged as large/risky.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLX-C1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C: Code Modification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generate diffs, not full-file rewrites</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a developer, I want the agent to generate a code diff (not full-file rewrites), so that changes are minimal and reviewable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Output is a unified diff/patch, not a full file replacement, except when creating new files.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">epic:code-modification, priority:must, type:feature, phase:1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLX-C2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Write/update tests alongside changes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a developer, I want the agent to write or update tests alongside code changes, so that the change is verifiable and future-proof.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For any behavior change, at least one corresponding test is added or updated.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">epic:code-modification, priority:should, type:feature, phase:1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLX-C3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run test suite after edits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a developer, I want the agent to run the existing test suite after making changes, so that regressions are caught immediately.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test suite runs automatically post-edit; results (pass/fail + output) are captured.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLX-C4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retry and self-correct on failure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a developer, I want the agent to retry and self-correct when tests fail, so that I don't have to manually debug its first attempt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">On failure, error output is fed back to the reasoning engine, which proposes a revised diff, up to a configurable retry limit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLX-D1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D: Human Oversight &amp; Trust</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deliver changes as pull requests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a tech lead, I want every agent change delivered as a pull request, so that a human always reviews before merge.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No commits land on protected branches without PR + approval flow.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">epic:human-oversight, priority:must, type:feature, phase:1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLX-D2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Show reasoning trace in PR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a reviewer, I want to see the agent's reasoning trace alongside the diff, so that I understand why it made each change.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PR description includes a summary of the plan, key decisions, and test results.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">epic:human-oversight, priority:should, type:feature, phase:1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLX-D3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accept conversational PR feedback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a developer, I want to reject or request changes to an agent's PR conversationally, so that I can course-correct without starting over.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feedback on a PR is fed back into the agent's context for a revised attempt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Could</t>
+  </si>
+  <si>
+    <t xml:space="preserve">epic:human-oversight, priority:could, type:feature, phase:1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLX-D4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Task outcomes dashboard (basic/CLI)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As an engineering manager, I want visibility into how many tasks the agent attempted, resolved, or failed, so that I can gauge its reliability over time.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A dashboard/log shows task outcomes, retry counts, and time-to-resolution.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">epic:human-oversight, priority:could, type:chore, phase:1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLX-E1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E: Safety &amp; Guardrails</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sandbox all code execution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a developer, I want the agent to run in a sandboxed environment, so that it can't affect my machine or production systems directly.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All code execution happens in an isolated container/VM with no access to host secrets or unrelated systems.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">epic:safety, priority:must, type:chore, phase:1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLX-E2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirm before destructive operations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a developer, I want the agent to ask for explicit confirmation before destructive operations, so that mistakes are never silent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Any operation on a configurable 'dangerous ops' list requires an explicit user confirmation step.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">epic:safety, priority:must, type:feature, phase:1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLX-E3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cap retries per task</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a developer, I want a hard cap on retries per task, so that a stuck task doesn't burn unbounded time or API cost.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configurable max retry count; task is marked 'needs human help' once exceeded, rather than looping forever.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLX-F1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F: Developer Experience</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Submit tasks via CLI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a developer, I want to submit a task via CLI, so that I can integrate this into my existing terminal workflow.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">`solvix run "&lt;task description&gt;"` triggers the full loop against the current repo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">epic:dev-experience, priority:must, type:feature, phase:1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLX-F2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Live progress updates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a developer, I want to see live progress (what file it's looking at, what it's trying), so that I'm not staring at a black box.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Streaming status updates during retrieval, planning, editing, and testing phases.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">epic:dev-experience, priority:should, type:feature, phase:1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLX-F3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configurable path allow/deny list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a developer, I want to configure which parts of the repo the agent is allowed to touch, so that sensitive files are never modified.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A config file (.solvix.yml) supports include/exclude paths, enforced before any write operation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLX-P2-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phase 2: Trust &amp; UX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G: Platform Integration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GitHub App integration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a developer, I want the agent to run as a GitHub App that responds to issues/PR comments, so that I don't need the CLI to trigger tasks.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Installing the GitHub App on a repo allows triggering tasks via issue labels or comments; agent posts PRs automatically without local CLI use.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">epic:platform-integration, priority:must, type:feature, phase:2</t>
+  </si>
+  <si>
     <t xml:space="preserve">To Do</t>
   </si>
   <si>
-    <t xml:space="preserve">SLX-B3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Produce a reviewable task plan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a tech lead, I want the agent to break a larger requirement into a task plan I can review before it starts editing, so that I can catch scope issues early.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Agent outputs an ordered plan (files to touch, approach) before any code is modified, and waits for approval if the task is flagged as large/risky.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLX-C1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C: Code Modification</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generate diffs, not full-file rewrites</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a developer, I want the agent to generate a code diff (not full-file rewrites), so that changes are minimal and reviewable.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Output is a unified diff/patch, not a full file replacement, except when creating new files.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">epic:code-modification, priority:must, type:feature, phase:1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLX-C2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sprint 7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Write/update tests alongside changes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a developer, I want the agent to write or update tests alongside code changes, so that the change is verifiable and future-proof.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">For any behavior change, at least one corresponding test is added or updated.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">epic:code-modification, priority:should, type:feature, phase:1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLX-C3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sprint 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Run test suite after edits</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a developer, I want the agent to run the existing test suite after making changes, so that regressions are caught immediately.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test suite runs automatically post-edit; results (pass/fail + output) are captured.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLX-C4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Retry and self-correct on failure</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a developer, I want the agent to retry and self-correct when tests fail, so that I don't have to manually debug its first attempt.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">On failure, error output is fed back to the reasoning engine, which proposes a revised diff, up to a configurable retry limit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLX-D1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D: Human Oversight &amp; Trust</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sprint 6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deliver changes as pull requests</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a tech lead, I want every agent change delivered as a pull request, so that a human always reviews before merge.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No commits land on protected branches without PR + approval flow.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">epic:human-oversight, priority:must, type:feature, phase:1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLX-D2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Show reasoning trace in PR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a reviewer, I want to see the agent's reasoning trace alongside the diff, so that I understand why it made each change.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PR description includes a summary of the plan, key decisions, and test results.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">epic:human-oversight, priority:should, type:feature, phase:1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLX-D3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Accept conversational PR feedback</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a developer, I want to reject or request changes to an agent's PR conversationally, so that I can course-correct without starting over.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Feedback on a PR is fed back into the agent's context for a revised attempt.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Could</t>
-  </si>
-  <si>
-    <t xml:space="preserve">epic:human-oversight, priority:could, type:feature, phase:1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLX-D4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Task outcomes dashboard (basic/CLI)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As an engineering manager, I want visibility into how many tasks the agent attempted, resolved, or failed, so that I can gauge its reliability over time.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A dashboard/log shows task outcomes, retry counts, and time-to-resolution.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">epic:human-oversight, priority:could, type:chore, phase:1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLX-E1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E: Safety &amp; Guardrails</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sprint 5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sandbox all code execution</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a developer, I want the agent to run in a sandboxed environment, so that it can't affect my machine or production systems directly.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All code execution happens in an isolated container/VM with no access to host secrets or unrelated systems.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">epic:safety, priority:must, type:chore, phase:1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLX-E2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirm before destructive operations</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a developer, I want the agent to ask for explicit confirmation before destructive operations, so that mistakes are never silent.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Any operation on a configurable 'dangerous ops' list requires an explicit user confirmation step.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">epic:safety, priority:must, type:feature, phase:1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLX-E3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cap retries per task</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a developer, I want a hard cap on retries per task, so that a stuck task doesn't burn unbounded time or API cost.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Configurable max retry count; task is marked 'needs human help' once exceeded, rather than looping forever.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLX-F1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F: Developer Experience</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Submit tasks via CLI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a developer, I want to submit a task via CLI, so that I can integrate this into my existing terminal workflow.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">`solvix run "&lt;task description&gt;"` triggers the full loop against the current repo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">epic:dev-experience, priority:must, type:feature, phase:1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLX-F2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Live progress updates</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a developer, I want to see live progress (what file it's looking at, what it's trying), so that I'm not staring at a black box.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Streaming status updates during retrieval, planning, editing, and testing phases.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">epic:dev-experience, priority:should, type:feature, phase:1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLX-F3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Configurable path allow/deny list</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a developer, I want to configure which parts of the repo the agent is allowed to touch, so that sensitive files are never modified.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A config file (.solvix.yml) supports include/exclude paths, enforced before any write operation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLX-P2-1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phase 2: Trust &amp; UX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G: Platform Integration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sprint 9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GitHub App integration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">As a developer, I want the agent to run as a GitHub App that responds to issues/PR comments, so that I don't need the CLI to trigger tasks.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Installing the GitHub App on a repo allows triggering tasks via issue labels or comments; agent posts PRs automatically without local CLI use.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">epic:platform-integration, priority:must, type:feature, phase:2</t>
-  </si>
-  <si>
     <t xml:space="preserve">SLX-P2-2</t>
   </si>
   <si>
@@ -681,7 +681,46 @@
     <t xml:space="preserve">As a developer, I want an interactive mode where the agent proposes one diff at a time directly against my real working files (not a sandboxed scratch copy ending in a PR), so that I can review and approve changes live, similar to working with a pair-programming assistant.</t>
   </si>
   <si>
-    <t xml:space="preserve">Running  reads the repo the same way as , but proposes each diff directly against the real working tree one step at a time, waits for explicit per-diff approval before writing it, and does not require a full task to complete before any change is visible — this is an additive mode alongside the existing sandboxed, PR-based  flow, not a replacement for it.</t>
+    <t xml:space="preserve">Running solvix chat reads the repo the same way as solvix run, but proposes each diff directly against the real working tree one step at a time, waits for explicit per-diff approval before writing it, and does not require a full task to complete before any change is visible — this is an additive mode alongside the existing sandboxed, PR-based solvix run flow, not a replacement for it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLX-C5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Detect assertion-gaming on retry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a developer, I want the system to flag (not just silently accept) a retry that passes tests by rewriting an expected/literal value in a test assertion rather than fixing the implementation, so that a locally-run smaller model cannot satisfy "tests pass" by rewriting the test to match whatever the code already does.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Given a retry attempt whose diff modifies a literal/expected value inside an existing or newly-added assertion (e.g. a hardcoded number, string, or comparison target) in the same step where the previous attempt failed specifically because of that literal, the step result flags this explicitly (e.g. assertion_literal_changed=True with the before/after values) even if the test suite ultimately passes — verified with a case reproducing the real add(0.1, 0.2) == 0.3 -&gt; == 0.30000000000000004 example found during SLX-D2's smoke test.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">epic:code-modification, priority:should, type:bug, phase:1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLX-C6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feed diff-generation failures into the outer retry loop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a developer, I want a DiffGenerationError (raised after propose_diff exhausts its own internal one-shot correction retry) to consume one attempt of the outer per-step retry budget rather than immediately terminating the step with needs_human_help=True, so that a malformed/unparseable diff gets the same real retry opportunity a failed test already gets, instead of wasting unused attempts and forcing a manual full re-run.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Given a step whose first propose_diff call raises DiffGenerationError, execute_step_with_verification treats this as a normal retriable failure within its own outer per-step budget (max_retries) — feeding the parse/diff-generation failure reason into the next attempt's prompt, the same way a test failure's output is fed back today — and only sets needs_human_help=True once the OUTER budget itself is exhausted, not on the first DiffGenerationError. Reproduced by the real missing ---/+++ header case found live during SLX-F2's smoke test.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLX-C7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Detect tolerance/rounding-wrapper assertion-gaming</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As a developer, I want the system to also flag a retry that makes a failing assertion pass by wrapping the comparison in a tolerance/rounding mechanism (round(), pytest.approx, abs(x-y)&lt;epsilon, or similar) rather than fixing the implementation, so that this style of gaming — found during SLX-C5's smoke test to be this model's more common default cheating behavior, more common than the literal-value swap SLX-C5 already catches — does not silently pass undetected.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Given a retry attempt whose diff introduces a tolerance/rounding wrapper (round(), pytest.approx, math.isclose, or an inline absolute-difference-under-epsilon pattern) around a comparison in the same assertion where the previous attempt failed on an exact-equality check, the step result flags this explicitly (with the before/after assertion text), even if the test suite ultimately passes — reusing SLX-C5's existing assertion_gaming_suspected/assertion_gaming_details fields and "Needs attention" PR surfacing rather than inventing a new mechanism.</t>
   </si>
   <si>
     <t xml:space="preserve">Focus</t>
@@ -1263,7 +1302,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K41"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
@@ -1485,12 +1524,12 @@
         <v>47</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>48</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>12</v>
@@ -1502,13 +1541,13 @@
         <v>23</v>
       </c>
       <c r="E7" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="G7" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>52</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>18</v>
@@ -1525,25 +1564,25 @@
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>53</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>54</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>28</v>
       </c>
       <c r="E8" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="G8" s="3" t="s">
         <v>56</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>57</v>
       </c>
       <c r="H8" s="5" t="s">
         <v>18</v>
@@ -1552,7 +1591,7 @@
         <v>19</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K8" s="3" t="s">
         <v>21</v>
@@ -1560,25 +1599,25 @@
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="D9" s="3" t="s">
+      <c r="E9" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="F9" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="G9" s="3" t="s">
         <v>62</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>63</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>32</v>
@@ -1587,33 +1626,33 @@
         <v>19</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>48</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="D10" s="3" t="s">
+      <c r="E10" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="F10" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="G10" s="3" t="s">
         <v>68</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>69</v>
       </c>
       <c r="H10" s="5" t="s">
         <v>18</v>
@@ -1622,7 +1661,7 @@
         <v>33</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K10" s="3" t="s">
         <v>21</v>
@@ -1630,25 +1669,25 @@
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="E11" s="3" t="s">
+      <c r="F11" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="G11" s="3" t="s">
         <v>72</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>73</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>18</v>
@@ -1657,7 +1696,7 @@
         <v>19</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K11" s="3" t="s">
         <v>21</v>
@@ -1665,25 +1704,25 @@
     </row>
     <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" s="3" t="s">
+      <c r="D12" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="E12" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="F12" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="G12" s="3" t="s">
         <v>78</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>79</v>
       </c>
       <c r="H12" s="5" t="s">
         <v>18</v>
@@ -1692,33 +1731,33 @@
         <v>33</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>48</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="E13" s="3" t="s">
+      <c r="F13" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="G13" s="3" t="s">
         <v>83</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>84</v>
       </c>
       <c r="H13" s="6" t="s">
         <v>32</v>
@@ -1727,103 +1766,103 @@
         <v>33</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>48</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>12</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>43</v>
       </c>
       <c r="E14" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F14" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="G14" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="H14" s="7" t="s">
         <v>89</v>
-      </c>
-      <c r="H14" s="7" t="s">
-        <v>90</v>
       </c>
       <c r="I14" s="3" t="s">
         <v>19</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>48</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>12</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>43</v>
       </c>
       <c r="E15" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="F15" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="G15" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="G15" s="3" t="s">
-        <v>95</v>
-      </c>
       <c r="H15" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I15" s="3" t="s">
         <v>33</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>48</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C16" s="3" t="s">
+      <c r="D16" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="E16" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="F16" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="G16" s="3" t="s">
         <v>101</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>102</v>
       </c>
       <c r="H16" s="5" t="s">
         <v>18</v>
@@ -1832,7 +1871,7 @@
         <v>19</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K16" s="3" t="s">
         <v>21</v>
@@ -1840,25 +1879,25 @@
     </row>
     <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E17" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="B17" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="E17" s="3" t="s">
+      <c r="F17" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="G17" s="3" t="s">
         <v>106</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>107</v>
       </c>
       <c r="H17" s="5" t="s">
         <v>18</v>
@@ -1867,7 +1906,7 @@
         <v>33</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K17" s="3" t="s">
         <v>21</v>
@@ -1875,25 +1914,25 @@
     </row>
     <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E18" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="E18" s="3" t="s">
+      <c r="F18" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="G18" s="3" t="s">
         <v>111</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>112</v>
       </c>
       <c r="H18" s="5" t="s">
         <v>18</v>
@@ -1902,7 +1941,7 @@
         <v>40</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K18" s="3" t="s">
         <v>21</v>
@@ -1910,25 +1949,25 @@
     </row>
     <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C19" s="3" t="s">
+      <c r="D19" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="E19" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="D19" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="E19" s="3" t="s">
+      <c r="F19" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="F19" s="3" t="s">
+      <c r="G19" s="3" t="s">
         <v>116</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>117</v>
       </c>
       <c r="H19" s="5" t="s">
         <v>18</v>
@@ -1937,7 +1976,7 @@
         <v>40</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K19" s="3" t="s">
         <v>21</v>
@@ -1945,25 +1984,25 @@
     </row>
     <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="E20" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="E20" s="3" t="s">
+      <c r="F20" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="G20" s="3" t="s">
         <v>121</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>122</v>
       </c>
       <c r="H20" s="6" t="s">
         <v>32</v>
@@ -1972,33 +2011,33 @@
         <v>33</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>48</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E21" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="B21" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="E21" s="3" t="s">
+      <c r="F21" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="F21" s="3" t="s">
+      <c r="G21" s="3" t="s">
         <v>126</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>127</v>
       </c>
       <c r="H21" s="5" t="s">
         <v>18</v>
@@ -2007,7 +2046,7 @@
         <v>40</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K21" s="3" t="s">
         <v>21</v>
@@ -2015,37 +2054,37 @@
     </row>
     <row r="22" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="B22" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="C22" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="D22" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="E22" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="F22" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="G22" s="3" t="s">
         <v>133</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>134</v>
       </c>
       <c r="H22" s="5" t="s">
         <v>18</v>
       </c>
       <c r="I22" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="J22" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="J22" s="3" t="s">
+      <c r="K22" s="3" t="s">
         <v>136</v>
-      </c>
-      <c r="K22" s="3" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2053,13 +2092,13 @@
         <v>137</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>138</v>
@@ -2080,7 +2119,7 @@
         <v>141</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>48</v>
+        <v>136</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2088,10 +2127,10 @@
         <v>142</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>143</v>
@@ -2109,13 +2148,13 @@
         <v>18</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="J24" s="3" t="s">
         <v>147</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>48</v>
+        <v>136</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2123,7 +2162,7 @@
         <v>148</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>13</v>
@@ -2150,7 +2189,7 @@
         <v>152</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>48</v>
+        <v>136</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2158,10 +2197,10 @@
         <v>153</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>154</v>
@@ -2176,7 +2215,7 @@
         <v>157</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I26" s="3" t="s">
         <v>19</v>
@@ -2185,7 +2224,7 @@
         <v>158</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>48</v>
+        <v>136</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2193,10 +2232,10 @@
         <v>159</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>154</v>
@@ -2211,7 +2250,7 @@
         <v>162</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I27" s="3" t="s">
         <v>33</v>
@@ -2220,7 +2259,7 @@
         <v>163</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>48</v>
+        <v>136</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2228,10 +2267,10 @@
         <v>164</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>165</v>
@@ -2249,13 +2288,13 @@
         <v>32</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="J28" s="3" t="s">
         <v>141</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>48</v>
+        <v>136</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2284,13 +2323,13 @@
         <v>18</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="J29" s="3" t="s">
         <v>176</v>
       </c>
       <c r="K29" s="3" t="s">
-        <v>48</v>
+        <v>136</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2325,7 +2364,7 @@
         <v>176</v>
       </c>
       <c r="K30" s="3" t="s">
-        <v>48</v>
+        <v>136</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2351,16 +2390,16 @@
         <v>185</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="J31" s="3" t="s">
         <v>186</v>
       </c>
       <c r="K31" s="3" t="s">
-        <v>48</v>
+        <v>136</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2389,13 +2428,13 @@
         <v>32</v>
       </c>
       <c r="I32" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="J32" s="3" t="s">
         <v>191</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>48</v>
+        <v>136</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2421,7 +2460,7 @@
         <v>196</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I33" s="3" t="s">
         <v>19</v>
@@ -2430,7 +2469,7 @@
         <v>186</v>
       </c>
       <c r="K33" s="3" t="s">
-        <v>48</v>
+        <v>136</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2441,7 +2480,7 @@
         <v>170</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>193</v>
@@ -2465,7 +2504,7 @@
         <v>201</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>48</v>
+        <v>136</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2500,7 +2539,7 @@
         <v>34</v>
       </c>
       <c r="K35" s="3" t="s">
-        <v>48</v>
+        <v>136</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2535,7 +2574,7 @@
         <v>34</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>48</v>
+        <v>136</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2546,10 +2585,10 @@
         <v>12</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>211</v>
@@ -2570,10 +2609,10 @@
         <v>214</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
         <v>215</v>
       </c>
@@ -2596,20 +2635,125 @@
         <v>218</v>
       </c>
       <c r="H38" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="I38" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="J38" s="3" t="s">
         <v>186</v>
       </c>
       <c r="K38" s="3" t="s">
-        <v>48</v>
+        <v>136</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="G39" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="H39" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="I39" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J39" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="K39" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="G40" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="H40" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="I40" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="J40" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="K40" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="113.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="H41" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="I41" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J41" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="K41" s="3" t="s">
+        <v>136</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K38"/>
+  <autoFilter ref="A1:K41"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2644,13 +2788,13 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>219</v>
+        <v>232</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>220</v>
+        <v>233</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>221</v>
+        <v>234</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2661,7 +2805,7 @@
         <v>12</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>222</v>
+        <v>235</v>
       </c>
       <c r="D2" s="3" t="n">
         <f aca="false">COUNTIF(Backlog!D:D,A2)</f>
@@ -2680,7 +2824,7 @@
         <v>12</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>223</v>
+        <v>236</v>
       </c>
       <c r="D3" s="3" t="n">
         <f aca="false">COUNTIF(Backlog!D:D,A3)</f>
@@ -2699,7 +2843,7 @@
         <v>12</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="D4" s="3" t="n">
         <f aca="false">COUNTIF(Backlog!D:D,A4)</f>
@@ -2712,13 +2856,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>12</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>225</v>
+        <v>238</v>
       </c>
       <c r="D5" s="3" t="n">
         <f aca="false">COUNTIF(Backlog!D:D,A5)</f>
@@ -2731,13 +2875,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>12</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="D6" s="3" t="n">
         <f aca="false">COUNTIF(Backlog!D:D,A6)</f>
@@ -2750,13 +2894,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
       <c r="D7" s="3" t="n">
         <f aca="false">COUNTIF(Backlog!D:D,A7)</f>
@@ -2769,17 +2913,17 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>228</v>
+        <v>241</v>
       </c>
       <c r="D8" s="3" t="n">
         <f aca="false">COUNTIF(Backlog!D:D,A8)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E8" s="3" t="n">
         <f aca="false">SUMIF(Backlog!D:D,A8,Backlog!I:I)</f>
@@ -2794,7 +2938,7 @@
         <v>12</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>229</v>
+        <v>242</v>
       </c>
       <c r="D9" s="3" t="n">
         <f aca="false">COUNTIF(Backlog!D:D,A9)</f>
@@ -2807,13 +2951,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="D10" s="3" t="n">
         <f aca="false">COUNTIF(Backlog!D:D,A10)</f>
@@ -2829,10 +2973,10 @@
         <v>143</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>231</v>
+        <v>244</v>
       </c>
       <c r="D11" s="3" t="n">
         <f aca="false">COUNTIF(Backlog!D:D,A11)</f>
@@ -2848,10 +2992,10 @@
         <v>154</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>232</v>
+        <v>245</v>
       </c>
       <c r="D12" s="3" t="n">
         <f aca="false">COUNTIF(Backlog!D:D,A12)</f>
@@ -2867,7 +3011,7 @@
         <v>165</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>166</v>
@@ -2889,7 +3033,7 @@
         <v>170</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>233</v>
+        <v>246</v>
       </c>
       <c r="D14" s="3" t="n">
         <f aca="false">COUNTIF(Backlog!D:D,A14)</f>
@@ -2908,7 +3052,7 @@
         <v>170</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>234</v>
+        <v>247</v>
       </c>
       <c r="D15" s="3" t="n">
         <f aca="false">COUNTIF(Backlog!D:D,A15)</f>
@@ -2927,7 +3071,7 @@
         <v>170</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>235</v>
+        <v>248</v>
       </c>
       <c r="D16" s="3" t="n">
         <f aca="false">COUNTIF(Backlog!D:D,A16)</f>
@@ -2940,13 +3084,13 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>236</v>
+        <v>249</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
       <c r="D17" s="10" t="n">
         <f aca="false">SUM(D2:D16)</f>
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E17" s="10" t="n">
         <f aca="false">SUM(E2:E16)</f>
@@ -2981,10 +3125,10 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>220</v>
+        <v>233</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>221</v>
+        <v>234</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>18</v>
@@ -2993,7 +3137,7 @@
         <v>32</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3002,7 +3146,7 @@
       </c>
       <c r="B2" s="3" t="n">
         <f aca="false">COUNTIF(Backlog!B:B,A2)</f>
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C2" s="3" t="n">
         <f aca="false">SUMIF(Backlog!B:B,A2,Backlog!I:I)</f>
@@ -3014,7 +3158,7 @@
       </c>
       <c r="E2" s="3" t="n">
         <f aca="false">COUNTIFS(Backlog!B:B,A2,Backlog!H:H,"Should")</f>
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F2" s="3" t="n">
         <f aca="false">COUNTIFS(Backlog!B:B,A2,Backlog!H:H,"Could")</f>
@@ -3023,7 +3167,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B3" s="3" t="n">
         <f aca="false">COUNTIF(Backlog!B:B,A3)</f>
@@ -3073,11 +3217,11 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>236</v>
+        <v>249</v>
       </c>
       <c r="B5" s="10" t="n">
         <f aca="false">SUM(B2:B4)</f>
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C5" s="10" t="n">
         <f aca="false">SUM(C2:C4)</f>
@@ -3089,7 +3233,7 @@
       </c>
       <c r="E5" s="10" t="n">
         <f aca="false">SUM(E2:E4)</f>
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F5" s="10" t="n">
         <f aca="false">SUM(F2:F4)</f>

</xml_diff>